<commit_message>
Add Studio 5000 V32 rung comment import from the 91026 printout
Emit a Tags and Logic Comments CSV (and a review workbook) so every
converted Airknife rung gets a comment starting with GE Rung N. When the
Logicmaster printout had a rung comment, that text is included. Comments
are attached to the following printed rung, matching GE print order.

Co-authored-by: Jack Wren <K4VR@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/AIRKNIFE_vs_91026_differences.xlsx
+++ b/reports/AIRKNIFE_vs_91026_differences.xlsx
@@ -1231,7 +1231,11 @@
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J4" s="9" t="inlineStr"/>
       <c r="K4" s="9" t="inlineStr"/>
     </row>
@@ -1303,11 +1307,7 @@
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
     </row>
@@ -1343,7 +1343,11 @@
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
     </row>
@@ -1631,11 +1635,7 @@
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
     </row>
@@ -1677,7 +1677,11 @@
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
     </row>
@@ -1705,7 +1709,7 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -1732,16 +1736,8 @@
 |                                +-----+                 +-----+</t>
         </is>
       </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J17" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE AUTO AND MANUAL BLOWER SPEED INPUTS ARE SCALED TO 0-4095 IN THE ) ( CONFIGUATION FOR THE ANALOG INPUT CARD. ) ( )</t>
-        </is>
-      </c>
+      <c r="I17" s="13" t="inlineStr"/>
+      <c r="J17" s="13" t="inlineStr"/>
       <c r="K17" s="13" t="n">
         <v>0.966</v>
       </c>
@@ -1770,7 +1766,7 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
@@ -1797,16 +1793,8 @@
 |                                +-----+                 +-----+</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE NEXT GROUP OF RUNGS CONTROL INDICATOR LIGHTS. ) ( )</t>
-        </is>
-      </c>
+      <c r="I18" s="13" t="inlineStr"/>
+      <c r="J18" s="13" t="inlineStr"/>
       <c r="K18" s="13" t="n">
         <v>0.977</v>
       </c>
@@ -1979,7 +1967,7 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>( ) ( DOWN SLOW ROTATION IS ALLOWED FROM 0 THRU 25 DEGREES, 170 THRU ) ( 205 DEGREES, 350 THRU 360 DEGREES OR ANYWHERE ABOVE MID-POSITION. ) ( )</t>
+          <t>( ) ( UP FAST ROTATION IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
         </is>
       </c>
       <c r="K21" s="13" t="n">
@@ -2010,7 +1998,7 @@
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
@@ -2027,8 +2015,16 @@
 *       +-----------------------+</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
-      <c r="J22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( DOWN FAST IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
+        </is>
+      </c>
       <c r="K22" s="13" t="n">
         <v>0.8149999999999999</v>
       </c>
@@ -2081,7 +2077,7 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>( ) ( DOWN SLOW ROTATION IS ALLOWED FROM 0 THRU 25 DEGREES, 170 THRU 205 ) ( DEGREES, 350 THRU 360 DEGREES OR ANYWHERE ABOVE THE ELEVATOR ) ( MID-POSITION. ) ( )</t>
+          <t>( ) ( UP FAST IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES DISENGAGED. ) ( )</t>
         </is>
       </c>
       <c r="K23" s="13" t="n">
@@ -2112,7 +2108,7 @@
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
@@ -2129,8 +2125,16 @@
 *       +-----------------------+</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr"/>
-      <c r="J24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( DOWN FAST IS ONLY ALLOWED ABOVE THE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
+        </is>
+      </c>
       <c r="K24" s="13" t="n">
         <v>0.8149999999999999</v>
       </c>
@@ -2183,7 +2187,11 @@
         </is>
       </c>
       <c r="I25" s="16" t="inlineStr"/>
-      <c r="J25" s="16" t="inlineStr"/>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS DETERMINE THE MODE OF THE KNIFE HORIZONTAL ) ( POSITIONERS. ) ( )</t>
+        </is>
+      </c>
       <c r="K25" s="16" t="inlineStr"/>
     </row>
     <row r="26" ht="30" customHeight="1">
@@ -2414,7 +2422,7 @@
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
@@ -2438,16 +2446,8 @@
 *--] [--+</t>
         </is>
       </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( Use Gap Auto to only allow movement if the correct mode from ACT ) ( is on. ) ( ) ( Skew mode, Passline mode (temp. disabled 3/24/17, ATM mode, ) ( and Z-Assist mode. ) ( )</t>
-        </is>
-      </c>
+      <c r="I30" s="13" t="inlineStr"/>
+      <c r="J30" s="13" t="inlineStr"/>
       <c r="K30" s="13" t="n">
         <v>0.5659999999999999</v>
       </c>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>( ) ( Use height movement in Auto when ACT is in Height or Z-assist mode ) ( ) ( ) ( Use this timer to keep the Manual Request high for a time delay after ) ( swithcing back to auto. ) ( ) ( ) ( )</t>
+          <t>( ) ( Use Gap Auto to only allow movement if the correct mode from ACT ) ( is on. ) ( ) ( Skew mode, Passline mode (temp. disabled 3/24/17, ATM mode, ) ( and Z-Assist mode. ) ( )</t>
         </is>
       </c>
       <c r="K31" s="13" t="n">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>( ) ( Use this timer to pulse the moves for the knives in and out. ) ( This is to prevent overshoot and emulate how the operator ) ( bumps the knives in and out. ) ( ) ( ) ( Setpoint in 1st Timer, PULSEKN, %M0906 is the off delay (200 = 2secs) ) ( Setpoint in 2nd Timer, PULSKNR, %M0907 is the on time (25 = 250ms) ) ( )</t>
+          <t>( ) ( Use height movement in Auto when ACT is in Height or Z-assist mode ) ( ) ( ) ( Use this timer to keep the Manual Request high for a time delay after ) ( swithcing back to auto. ) ( ) ( ) ( )</t>
         </is>
       </c>
       <c r="K33" s="13" t="n">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE FRONT ) ( HORIZONTAL POSITIONERS. ) ( )</t>
+          <t>( ) ( AUTO MODE INDICATOR LIGHT CONTROL RELAYS. ) ( )</t>
         </is>
       </c>
       <c r="K34" s="13" t="n">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
@@ -2759,8 +2759,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr"/>
-      <c r="J35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE FRONT ) ( HORIZONTAL POSITIONERS. ) ( )</t>
+        </is>
+      </c>
       <c r="K35" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -2858,7 +2866,7 @@
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G37" s="15" t="inlineStr">
@@ -2885,16 +2893,8 @@
 *--] [-----] [----------+</t>
         </is>
       </c>
-      <c r="I37" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J37" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 1DR (FRONT KNIFE ) ( DRIVESIDE). ) ( )</t>
-        </is>
-      </c>
+      <c r="I37" s="13" t="inlineStr"/>
+      <c r="J37" s="13" t="inlineStr"/>
       <c r="K37" s="13" t="n">
         <v>0.968</v>
       </c>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G38" s="15" t="inlineStr">
@@ -2962,8 +2962,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I38" s="13" t="inlineStr"/>
-      <c r="J38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE OPERATOR SIDE FRONT ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K38" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -2992,7 +3000,7 @@
       </c>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G39" s="15" t="inlineStr">
@@ -3031,16 +3039,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I39" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J39" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED SELECT FOR 2MTR (OPERATOR SIDE FRONT HORIZONTAL). ) ( )</t>
-        </is>
-      </c>
+      <c r="I39" s="13" t="inlineStr"/>
+      <c r="J39" s="13" t="inlineStr"/>
       <c r="K39" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 2DR (OPERATOR SIDE FRONT ) ( KNIFE HORIZONTAL). ) ( )</t>
+          <t>( ) ( FAST SPEED SELECT FOR 2MTR (OPERATOR SIDE FRONT HORIZONTAL). ) ( )</t>
         </is>
       </c>
       <c r="K40" s="13" t="n">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G41" s="15" t="inlineStr">
@@ -3173,8 +3173,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I41" s="13" t="inlineStr"/>
-      <c r="J41" s="13" t="inlineStr"/>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE REAR KNIFE ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K41" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -3203,7 +3211,7 @@
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G42" s="15" t="inlineStr">
@@ -3242,16 +3250,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED CONTROL FOR 3MTR. ) ( )</t>
-        </is>
-      </c>
+      <c r="I42" s="13" t="inlineStr"/>
+      <c r="J42" s="13" t="inlineStr"/>
       <c r="K42" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE THR INTERFACE RELAYS FOR 3DR. ) ( )</t>
+          <t>( ) ( FAST SPEED CONTROL FOR 3MTR. ) ( )</t>
         </is>
       </c>
       <c r="K43" s="13" t="n">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F44" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G44" s="15" t="inlineStr">
@@ -3384,8 +3384,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I44" s="13" t="inlineStr"/>
-      <c r="J44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE OPERATOR SIDE REAR KNIFE ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K44" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -3414,7 +3422,7 @@
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G45" s="15" t="inlineStr">
@@ -3453,16 +3461,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I45" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J45" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED CONTROL OF 4MTR. ) ( )</t>
-        </is>
-      </c>
+      <c r="I45" s="13" t="inlineStr"/>
+      <c r="J45" s="13" t="inlineStr"/>
       <c r="K45" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 4DR (REAR KNIFE OPERATOR ) ( SIDE HORIZONTAL POSITIONER). ) ( )</t>
+          <t>( ) ( FAST SPEED CONTROL OF 4MTR. ) ( )</t>
         </is>
       </c>
       <c r="K46" s="13" t="n">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>Added: %M00541; Ladder wiring or constants also differ</t>
+          <t>Added: %M00541; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G47" s="15" t="inlineStr">
@@ -3592,8 +3592,16 @@
 *--] [--+</t>
         </is>
       </c>
-      <c r="I47" s="13" t="inlineStr"/>
-      <c r="J47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( STARTER FAULT INDICATOR LIGHT ON THE PUSHBUTTON PANEL. ) ( )</t>
+        </is>
+      </c>
       <c r="K47" s="13" t="n">
         <v>0.944</v>
       </c>
@@ -3653,7 +3661,7 @@
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>( ) ( WHEN A DISENGAGE PUSHBUTTON REQUEST IS SEEN IN AUTO MODE, AUTO MODE ) ( IS DISABLED (LOCKED OUT) UNTIL THE AUTO/MAN SELECTOR SWITCH IS TOGGLED ) ( OR A BAFFLE ENGAGE PUSHBUTTON IS PRESSED. BAFFLE REQUESTS FROM THE WELD ) ( TRACKING ARE IGNORED WHILE THIS RUNG IS TRUE. ) ( )</t>
+          <t>( ) ( RESET STARTER FAULTS ) ( )</t>
         </is>
       </c>
       <c r="K48" s="13" t="n">
@@ -3983,7 +3991,7 @@
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+; Comment text differs</t>
+          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+</t>
         </is>
       </c>
       <c r="G56" s="15" t="inlineStr">
@@ -4010,16 +4018,8 @@
 |      +9.055000 +-----+       -5.099500 +-----+</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( Determine Skew of Top Knives ) ( ) ( ) ( Determine Top Side knife to Knife distance ) ( )</t>
-        </is>
-      </c>
+      <c r="I56" s="13" t="inlineStr"/>
+      <c r="J56" s="13" t="inlineStr"/>
       <c r="K56" s="13" t="n">
         <v>0.998</v>
       </c>
@@ -4176,7 +4176,11 @@
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr"/>
-      <c r="I59" s="9" t="inlineStr"/>
+      <c r="I59" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J59" s="9" t="inlineStr"/>
       <c r="K59" s="9" t="inlineStr"/>
     </row>
@@ -4218,11 +4222,7 @@
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr"/>
-      <c r="I60" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT ) ( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I60" s="9" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr"/>
       <c r="K60" s="9" t="inlineStr"/>
     </row>
@@ -4495,7 +4495,11 @@
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr"/>
-      <c r="I66" s="9" t="inlineStr"/>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J66" s="9" t="inlineStr"/>
       <c r="K66" s="9" t="inlineStr"/>
     </row>
@@ -4621,11 +4625,7 @@
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr"/>
-      <c r="I69" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I69" s="9" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
       <c r="K69" s="9" t="inlineStr"/>
     </row>
@@ -4668,7 +4668,11 @@
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
-      <c r="I70" s="9" t="inlineStr"/>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J70" s="9" t="inlineStr"/>
       <c r="K70" s="9" t="inlineStr"/>
     </row>
@@ -4794,11 +4798,7 @@
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr"/>
-      <c r="I73" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I73" s="9" t="inlineStr"/>
       <c r="J73" s="9" t="inlineStr"/>
       <c r="K73" s="9" t="inlineStr"/>
     </row>
@@ -4841,7 +4841,11 @@
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr"/>
-      <c r="I74" s="9" t="inlineStr"/>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J74" s="9" t="inlineStr"/>
       <c r="K74" s="9" t="inlineStr"/>
     </row>
@@ -4967,11 +4971,7 @@
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr"/>
-      <c r="I77" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I77" s="9" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="9" t="inlineStr"/>
     </row>
@@ -5189,7 +5189,11 @@
         </is>
       </c>
       <c r="H82" s="11" t="inlineStr"/>
-      <c r="I82" s="9" t="inlineStr"/>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J82" s="9" t="inlineStr"/>
       <c r="K82" s="9" t="inlineStr"/>
     </row>
@@ -5231,11 +5235,7 @@
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr"/>
-      <c r="I83" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I83" s="9" t="inlineStr"/>
       <c r="J83" s="9" t="inlineStr"/>
       <c r="K83" s="9" t="inlineStr"/>
     </row>
@@ -5278,7 +5278,11 @@
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr"/>
-      <c r="I84" s="9" t="inlineStr"/>
+      <c r="I84" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J84" s="9" t="inlineStr"/>
       <c r="K84" s="9" t="inlineStr"/>
     </row>
@@ -5362,7 +5366,11 @@
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr"/>
-      <c r="I86" s="9" t="inlineStr"/>
+      <c r="I86" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J86" s="9" t="inlineStr"/>
       <c r="K86" s="9" t="inlineStr"/>
     </row>
@@ -5404,11 +5412,7 @@
         </is>
       </c>
       <c r="H87" s="11" t="inlineStr"/>
-      <c r="I87" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I87" s="9" t="inlineStr"/>
       <c r="J87" s="9" t="inlineStr"/>
       <c r="K87" s="9" t="inlineStr"/>
     </row>
@@ -5580,7 +5584,11 @@
         </is>
       </c>
       <c r="H91" s="11" t="inlineStr"/>
-      <c r="I91" s="9" t="inlineStr"/>
+      <c r="I91" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J91" s="9" t="inlineStr"/>
       <c r="K91" s="9" t="inlineStr"/>
     </row>
@@ -5782,11 +5790,7 @@
         </is>
       </c>
       <c r="H96" s="11" t="inlineStr"/>
-      <c r="I96" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I96" s="9" t="inlineStr"/>
       <c r="J96" s="9" t="inlineStr"/>
       <c r="K96" s="9" t="inlineStr"/>
     </row>
@@ -5830,7 +5834,11 @@
         </is>
       </c>
       <c r="H97" s="11" t="inlineStr"/>
-      <c r="I97" s="9" t="inlineStr"/>
+      <c r="I97" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J97" s="9" t="inlineStr"/>
       <c r="K97" s="9" t="inlineStr"/>
     </row>
@@ -6086,11 +6094,7 @@
         </is>
       </c>
       <c r="H103" s="11" t="inlineStr"/>
-      <c r="I103" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I103" s="9" t="inlineStr"/>
       <c r="J103" s="9" t="inlineStr"/>
       <c r="K103" s="9" t="inlineStr"/>
     </row>
@@ -6132,7 +6136,11 @@
         </is>
       </c>
       <c r="H104" s="11" t="inlineStr"/>
-      <c r="I104" s="9" t="inlineStr"/>
+      <c r="I104" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J104" s="9" t="inlineStr"/>
       <c r="K104" s="9" t="inlineStr"/>
     </row>
@@ -6349,11 +6357,7 @@
         </is>
       </c>
       <c r="H109" s="11" t="inlineStr"/>
-      <c r="I109" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I109" s="9" t="inlineStr"/>
       <c r="J109" s="9" t="inlineStr"/>
       <c r="K109" s="9" t="inlineStr"/>
     </row>
@@ -6389,7 +6393,11 @@
         </is>
       </c>
       <c r="H110" s="11" t="inlineStr"/>
-      <c r="I110" s="9" t="inlineStr"/>
+      <c r="I110" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J110" s="9" t="inlineStr"/>
       <c r="K110" s="9" t="inlineStr"/>
     </row>
@@ -6441,7 +6449,7 @@
       <c r="I111" s="13" t="inlineStr"/>
       <c r="J111" s="13" t="inlineStr">
         <is>
-          <t>( ) ( ACT Appendix B: Section 5.1.2 ) ( ) ( R00436-440 Next Coating Weight Designation ) ( mapped from Wonderware at R00586-590 ) ( ) ( ) ( 3/14/17 ) ( %R436-440 was being overwritten due to being defined twice in wonderware ) ( so ) ( ACT changed to %R496-500 ) ( )</t>
+          <t>( ) ( ACT Appendix 3.2.k.1.0.x ) ( Knife Positions from ACT ) ( ) ( Permissive to move Knives in Auto. When in CLC Operatiing Mode, ACT ) ( controls the Pressure. Then if the oter modes, Z-Assist, Passline, ) ( Skew and ATM mode are selected, then the Knives can be moved ) ( automatically. ) ( ) ( )</t>
         </is>
       </c>
       <c r="K111" s="13" t="n">
@@ -6480,11 +6488,7 @@
         </is>
       </c>
       <c r="H112" s="11" t="inlineStr"/>
-      <c r="I112" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I112" s="9" t="inlineStr"/>
       <c r="J112" s="9" t="inlineStr"/>
       <c r="K112" s="9" t="inlineStr"/>
     </row>
@@ -6512,7 +6516,7 @@
       </c>
       <c r="F113" s="13" t="inlineStr">
         <is>
-          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ</t>
+          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G113" s="15" t="inlineStr">
@@ -6539,8 +6543,16 @@
 |                +-----+</t>
         </is>
       </c>
-      <c r="I113" s="13" t="inlineStr"/>
-      <c r="J113" s="13" t="inlineStr"/>
+      <c r="I113" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J113" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( ACT Appendix B: Section 5.1.2 ) ( ) ( R00436-440 Next Coating Weight Designation ) ( mapped from Wonderware at R00586-590 ) ( ) ( ) ( 3/14/17 ) ( %R436-440 was being overwritten due to being defined twice in wonderware ) ( so ) ( ACT changed to %R496-500 ) ( )</t>
+        </is>
+      </c>
       <c r="K113" s="13" t="n">
         <v>0.5649999999999999</v>
       </c>
@@ -6740,7 +6752,7 @@
       </c>
       <c r="F117" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |</t>
+          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |; Comment text differs</t>
         </is>
       </c>
       <c r="G117" s="15" t="inlineStr">
@@ -6767,8 +6779,16 @@
 |                +-----+                                 +-----+</t>
         </is>
       </c>
-      <c r="I117" s="13" t="inlineStr"/>
-      <c r="J117" s="13" t="inlineStr"/>
+      <c r="I117" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J117" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( ) ( ) ( Auto Mode Parameters based on Setpoints from ACT ) ( ) ( ) ( )</t>
+        </is>
+      </c>
       <c r="K117" s="13" t="n">
         <v>0.992</v>
       </c>
@@ -7793,7 +7813,11 @@
         </is>
       </c>
       <c r="H135" s="11" t="inlineStr"/>
-      <c r="I135" s="9" t="inlineStr"/>
+      <c r="I135" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J135" s="9" t="inlineStr"/>
       <c r="K135" s="9" t="inlineStr"/>
     </row>
@@ -7837,11 +7861,7 @@
         </is>
       </c>
       <c r="H136" s="11" t="inlineStr"/>
-      <c r="I136" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I136" s="9" t="inlineStr"/>
       <c r="J136" s="9" t="inlineStr"/>
       <c r="K136" s="9" t="inlineStr"/>
     </row>
@@ -7886,7 +7906,11 @@
         </is>
       </c>
       <c r="H137" s="11" t="inlineStr"/>
-      <c r="I137" s="9" t="inlineStr"/>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J137" s="9" t="inlineStr"/>
       <c r="K137" s="9" t="inlineStr"/>
     </row>
@@ -8102,11 +8126,7 @@
         </is>
       </c>
       <c r="H142" s="11" t="inlineStr"/>
-      <c r="I142" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I142" s="9" t="inlineStr"/>
       <c r="J142" s="9" t="inlineStr"/>
       <c r="K142" s="9" t="inlineStr"/>
     </row>
@@ -8142,7 +8162,11 @@
         </is>
       </c>
       <c r="H143" s="11" t="inlineStr"/>
-      <c r="I143" s="9" t="inlineStr"/>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J143" s="9" t="inlineStr"/>
       <c r="K143" s="9" t="inlineStr"/>
     </row>
@@ -9114,11 +9138,7 @@
         </is>
       </c>
       <c r="H170" s="11" t="inlineStr"/>
-      <c r="I170" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I170" s="9" t="inlineStr"/>
       <c r="J170" s="9" t="inlineStr"/>
       <c r="K170" s="9" t="inlineStr"/>
     </row>
@@ -9598,7 +9618,11 @@
           <t>coil BLOWENA</t>
         </is>
       </c>
-      <c r="G17" s="25" t="inlineStr"/>
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="n">
@@ -9652,11 +9676,7 @@
           <t>coil CR14</t>
         </is>
       </c>
-      <c r="G19" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G19" s="25" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="23" t="n">
@@ -9683,7 +9703,11 @@
           <t>coil BDRVFLT; fn ONDTR</t>
         </is>
       </c>
-      <c r="G20" s="25" t="inlineStr"/>
+      <c r="G20" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="n">
@@ -9849,7 +9873,7 @@
       </c>
       <c r="G26" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9902,11 @@
           <t>coil %M00929; fn SUB, GE</t>
         </is>
       </c>
-      <c r="G27" s="25" t="inlineStr"/>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="23" t="n">
@@ -9961,7 +9989,7 @@
       </c>
       <c r="G30" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -9990,7 +10018,11 @@
           <t>coil PB33-L</t>
         </is>
       </c>
-      <c r="G31" s="25" t="inlineStr"/>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="23" t="n">
@@ -10241,11 +10273,7 @@
           <t>coil SS6-L, SS9-L</t>
         </is>
       </c>
-      <c r="G40" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G40" s="25" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="23" t="n">
@@ -10272,7 +10300,11 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G41" s="25" t="inlineStr"/>
+      <c r="G41" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="n">
@@ -10461,11 +10493,7 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G48" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G48" s="25" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="23" t="n">
@@ -10492,7 +10520,11 @@
           <t>fn MOVE, ADD, SUB</t>
         </is>
       </c>
-      <c r="G49" s="25" t="inlineStr"/>
+      <c r="G49" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="23" t="n">
@@ -11599,11 +11631,7 @@
           <t>coil RKRDRVF</t>
         </is>
       </c>
-      <c r="G90" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G90" s="25" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="23" t="n">
@@ -11630,7 +11658,11 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G91" s="25" t="inlineStr"/>
+      <c r="G91" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="23" t="n">
@@ -11657,11 +11689,7 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G92" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G92" s="25" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="23" t="n">
@@ -11812,7 +11840,11 @@
           <t>*fn MUL, DIV</t>
         </is>
       </c>
-      <c r="G97" s="25" t="inlineStr"/>
+      <c r="G97" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="23" t="n">
@@ -11839,11 +11871,7 @@
           <t>*fn MUL, DIV</t>
         </is>
       </c>
-      <c r="G98" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G98" s="25" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="23" t="n">
@@ -11870,7 +11898,11 @@
           <t>*coil LIM11; fn GT</t>
         </is>
       </c>
-      <c r="G99" s="25" t="inlineStr"/>
+      <c r="G99" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="23" t="n">
@@ -12059,11 +12091,7 @@
           <t>*coil XLIM41; fn GT</t>
         </is>
       </c>
-      <c r="G106" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G106" s="25" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="23" t="n">
@@ -12090,7 +12118,11 @@
           <t>*coil FZNCCWS</t>
         </is>
       </c>
-      <c r="G107" s="25" t="inlineStr"/>
+      <c r="G107" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="23" t="n">
@@ -12171,11 +12203,7 @@
           <t>*coil FZNCWF</t>
         </is>
       </c>
-      <c r="G110" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G110" s="25" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="23" t="n">
@@ -12297,7 +12325,7 @@
       </c>
       <c r="G114" s="29" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -12326,11 +12354,7 @@
           <t>*coil FKRFST</t>
         </is>
       </c>
-      <c r="G115" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G115" s="25" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="23" t="n">
@@ -12419,7 +12443,11 @@
           <t>*coil LIM12; fn GT</t>
         </is>
       </c>
-      <c r="G118" s="25" t="inlineStr"/>
+      <c r="G118" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="23" t="n">
@@ -12608,11 +12636,7 @@
           <t>*coil XLIM42; fn GT</t>
         </is>
       </c>
-      <c r="G125" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G125" s="25" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="23" t="n">
@@ -12639,7 +12663,11 @@
           <t>*coil RZNCWSL</t>
         </is>
       </c>
-      <c r="G126" s="25" t="inlineStr"/>
+      <c r="G126" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="23" t="n">
@@ -12720,11 +12748,7 @@
           <t>*coil RZNCCWF</t>
         </is>
       </c>
-      <c r="G129" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G129" s="25" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="23" t="n">
@@ -12846,7 +12870,7 @@
       </c>
       <c r="G133" s="29" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -12875,11 +12899,7 @@
           <t>*coil RKRFST</t>
         </is>
       </c>
-      <c r="G134" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G134" s="25" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="23" t="n">
@@ -13297,7 +13317,7 @@
       </c>
       <c r="G148" s="29" t="inlineStr">
         <is>
-          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -13417,7 +13437,11 @@
           <t>*coil %M00924</t>
         </is>
       </c>
-      <c r="G152" s="25" t="inlineStr"/>
+      <c r="G152" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="23" t="n">
@@ -13525,11 +13549,7 @@
           <t>*coil PULSKMR; fn ONDTR</t>
         </is>
       </c>
-      <c r="G156" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G156" s="25" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="26" t="n">
@@ -13589,7 +13609,7 @@
       </c>
       <c r="G158" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -13651,7 +13671,7 @@
       </c>
       <c r="G160" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -13680,7 +13700,11 @@
           <t>*coil FKDISLO</t>
         </is>
       </c>
-      <c r="G161" s="25" t="inlineStr"/>
+      <c r="G161" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="23" t="n">
@@ -13815,11 +13839,7 @@
           <t>*coil FKDBDIS</t>
         </is>
       </c>
-      <c r="G166" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G166" s="25" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="26" t="n">
@@ -13848,7 +13868,7 @@
       </c>
       <c r="G167" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -13879,7 +13899,7 @@
       </c>
       <c r="G168" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -13939,7 +13959,11 @@
           <t>*coil FKOISLO</t>
         </is>
       </c>
-      <c r="G170" s="25" t="inlineStr"/>
+      <c r="G170" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="23" t="n">
@@ -14074,11 +14098,7 @@
           <t>*coil FKOBDIS</t>
         </is>
       </c>
-      <c r="G175" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G175" s="25" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="23" t="n">
@@ -14138,7 +14158,7 @@
       </c>
       <c r="G177" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -14169,7 +14189,7 @@
       </c>
       <c r="G178" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -14229,7 +14249,11 @@
           <t>*coil RKDISLO</t>
         </is>
       </c>
-      <c r="G180" s="25" t="inlineStr"/>
+      <c r="G180" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="23" t="n">
@@ -14364,11 +14388,7 @@
           <t>*coil RKDBDIS</t>
         </is>
       </c>
-      <c r="G185" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G185" s="25" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="26" t="n">
@@ -14397,7 +14417,7 @@
       </c>
       <c r="G186" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -14428,7 +14448,7 @@
       </c>
       <c r="G187" s="29" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
     </row>
@@ -14488,7 +14508,11 @@
           <t>*coil RKOISLO</t>
         </is>
       </c>
-      <c r="G189" s="25" t="inlineStr"/>
+      <c r="G189" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="23" t="n">
@@ -14623,11 +14647,7 @@
           <t>*coil RKOBDIS</t>
         </is>
       </c>
-      <c r="G194" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G194" s="25" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="23" t="n">
@@ -14654,7 +14674,11 @@
           <t>*coil RKDRVEN</t>
         </is>
       </c>
-      <c r="G195" s="25" t="inlineStr"/>
+      <c r="G195" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="23" t="n">
@@ -14762,11 +14786,7 @@
           <t>*coil %M00581</t>
         </is>
       </c>
-      <c r="G199" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G199" s="25" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="23" t="n">
@@ -14793,7 +14813,11 @@
           <t>*coil ST7FWD</t>
         </is>
       </c>
-      <c r="G200" s="25" t="inlineStr"/>
+      <c r="G200" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="23" t="n">
@@ -14874,11 +14898,7 @@
           <t>*coil ST8REV</t>
         </is>
       </c>
-      <c r="G203" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G203" s="25" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="23" t="n">
@@ -14905,7 +14925,11 @@
           <t>*coil STFLT5; fn ONDTR</t>
         </is>
       </c>
-      <c r="G204" s="25" t="inlineStr"/>
+      <c r="G204" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="23" t="n">
@@ -14986,11 +15010,7 @@
           <t>*coil STFLT8; fn ONDTR</t>
         </is>
       </c>
-      <c r="G207" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G207" s="25" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="26" t="n">
@@ -15019,7 +15039,7 @@
       </c>
       <c r="G208" s="29" t="inlineStr">
         <is>
-          <t>Added: %M00541; Ladder wiring or constants also differ</t>
+          <t>Added: %M00541; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -15129,11 +15149,7 @@
           <t>*coil PB40-AL, PB40-L</t>
         </is>
       </c>
-      <c r="G212" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G212" s="25" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="26" t="n">
@@ -15191,7 +15207,11 @@
           <t>*coil ATLKOUT</t>
         </is>
       </c>
-      <c r="G214" s="25" t="inlineStr"/>
+      <c r="G214" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="23" t="n">
@@ -15218,11 +15238,7 @@
           <t>*coil DISBAFO</t>
         </is>
       </c>
-      <c r="G215" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G215" s="25" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="23" t="n">
@@ -15311,7 +15327,11 @@
           <t>*coil BAFDIS</t>
         </is>
       </c>
-      <c r="G218" s="25" t="inlineStr"/>
+      <c r="G218" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="23" t="n">
@@ -15365,11 +15385,7 @@
           <t>*coil UNKNOQ1</t>
         </is>
       </c>
-      <c r="G220" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G220" s="25" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="23" t="n">
@@ -15458,7 +15474,11 @@
           <t>*coil IL2, SS2-L</t>
         </is>
       </c>
-      <c r="G223" s="25" t="inlineStr"/>
+      <c r="G223" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="23" t="n">
@@ -15541,7 +15561,11 @@
           <t>coil ACT_HBT; fn ONDTR</t>
         </is>
       </c>
-      <c r="G226" s="25" t="inlineStr"/>
+      <c r="G226" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="23" t="n">
@@ -15796,11 +15820,7 @@
           <t>fn ADD, MUL</t>
         </is>
       </c>
-      <c r="G235" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G235" s="25" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="23" t="n">
@@ -15827,7 +15847,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G236" s="25" t="inlineStr"/>
+      <c r="G236" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="26" t="n">
@@ -15856,7 +15880,7 @@
       </c>
       <c r="G237" s="29" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+; Comment text differs</t>
+          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+</t>
         </is>
       </c>
     </row>
@@ -15916,7 +15940,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G239" s="25" t="inlineStr"/>
+      <c r="G239" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="23" t="n">
@@ -15943,11 +15971,7 @@
           <t>fn ADD, MUL</t>
         </is>
       </c>
-      <c r="G240" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G240" s="25" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="23" t="n">
@@ -15974,7 +15998,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G241" s="25" t="inlineStr"/>
+      <c r="G241" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="23" t="n">
@@ -16117,11 +16145,7 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G246" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G246" s="25" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="19" t="n">
@@ -16206,7 +16230,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G249" s="25" t="inlineStr"/>
+      <c r="G249" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="23" t="n">
@@ -16233,11 +16261,7 @@
           <t>fn SUB, MUL</t>
         </is>
       </c>
-      <c r="G250" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G250" s="25" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="23" t="n">
@@ -16264,7 +16288,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G251" s="25" t="inlineStr"/>
+      <c r="G251" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="23" t="n">
@@ -16291,11 +16319,7 @@
           <t>fn SUB, MUL</t>
         </is>
       </c>
-      <c r="G252" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G252" s="25" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="23" t="n">
@@ -16962,7 +16986,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G275" s="25" t="inlineStr"/>
+      <c r="G275" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="23" t="n">
@@ -16989,11 +17017,7 @@
           <t>fn ADD, MUL</t>
         </is>
       </c>
-      <c r="G276" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G276" s="25" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="23" t="n">
@@ -17020,7 +17044,11 @@
           <t>fn DIV, INT</t>
         </is>
       </c>
-      <c r="G277" s="25" t="inlineStr"/>
+      <c r="G277" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="23" t="n">
@@ -17047,11 +17075,7 @@
           <t>fn ADD, MUL</t>
         </is>
       </c>
-      <c r="G278" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G278" s="25" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="23" t="n">
@@ -17078,7 +17102,11 @@
           <t>fn ADD, DIV</t>
         </is>
       </c>
-      <c r="G279" s="25" t="inlineStr"/>
+      <c r="G279" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="23" t="n">
@@ -17159,11 +17187,7 @@
           <t>coil %M00579; fn LE, GE</t>
         </is>
       </c>
-      <c r="G282" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G282" s="25" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="19" t="n">
@@ -17308,7 +17332,7 @@
       </c>
       <c r="G287" s="25" t="inlineStr">
         <is>
-          <t>Comment text differs (logic identical)</t>
+          <t>Comment printed in 91026 (logic identical)</t>
         </is>
       </c>
     </row>
@@ -18124,7 +18148,7 @@
       </c>
       <c r="G315" s="29" t="inlineStr">
         <is>
-          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ</t>
+          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -18435,11 +18459,7 @@
           <t>coil BKD_SPL; fn LE, MOVE</t>
         </is>
       </c>
-      <c r="G326" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G326" s="25" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" s="26" t="n">
@@ -18468,7 +18488,7 @@
       </c>
       <c r="G327" s="29" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |</t>
+          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |; Comment text differs</t>
         </is>
       </c>
     </row>
@@ -18524,11 +18544,7 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G329" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G329" s="25" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" s="23" t="n">
@@ -18555,7 +18571,11 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G330" s="25" t="inlineStr"/>
+      <c r="G330" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="26" t="n">
@@ -18814,11 +18834,7 @@
           <t>fn LT, MOVE</t>
         </is>
       </c>
-      <c r="G339" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G339" s="25" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" s="23" t="n">
@@ -18845,7 +18861,11 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G340" s="25" t="inlineStr"/>
+      <c r="G340" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="26" t="n">
@@ -19104,11 +19124,7 @@
           <t>fn LT, MOVE</t>
         </is>
       </c>
-      <c r="G349" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G349" s="25" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" s="23" t="n">
@@ -19135,7 +19151,11 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G350" s="25" t="inlineStr"/>
+      <c r="G350" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="26" t="n">
@@ -19394,11 +19414,7 @@
           <t>fn LT, MOVE</t>
         </is>
       </c>
-      <c r="G359" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G359" s="25" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" s="23" t="n">
@@ -19425,7 +19441,11 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G360" s="25" t="inlineStr"/>
+      <c r="G360" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="26" t="n">
@@ -19873,11 +19893,7 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G376" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G376" s="25" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" s="23" t="n">
@@ -19935,7 +19951,11 @@
           <t>coil KHATUPL; fn GE</t>
         </is>
       </c>
-      <c r="G378" s="25" t="inlineStr"/>
+      <c r="G378" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="23" t="n">
@@ -19989,11 +20009,7 @@
           <t>fn LE, MOVE</t>
         </is>
       </c>
-      <c r="G380" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G380" s="25" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" s="23" t="n">
@@ -20051,7 +20067,11 @@
           <t>fn SUB</t>
         </is>
       </c>
-      <c r="G382" s="25" t="inlineStr"/>
+      <c r="G382" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="23" t="n">
@@ -20375,11 +20395,7 @@
           <t>coil %M00577; fn GE</t>
         </is>
       </c>
-      <c r="G394" s="25" t="inlineStr">
-        <is>
-          <t>Comment text differs (logic identical)</t>
-        </is>
-      </c>
+      <c r="G394" s="25" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" s="19" t="n">
@@ -21479,7 +21495,11 @@
           <t>fn MOVE</t>
         </is>
       </c>
-      <c r="G432" s="25" t="inlineStr"/>
+      <c r="G432" s="25" t="inlineStr">
+        <is>
+          <t>Comment text differs (logic identical)</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="23" t="n">
@@ -21906,7 +21926,11 @@
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J4" s="9" t="inlineStr"/>
       <c r="K4" s="9" t="inlineStr"/>
     </row>
@@ -21978,11 +22002,7 @@
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
     </row>
@@ -22018,7 +22038,11 @@
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
     </row>
@@ -22306,11 +22330,7 @@
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
     </row>
@@ -22352,7 +22372,11 @@
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
     </row>
@@ -22736,7 +22760,11 @@
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr"/>
-      <c r="I25" s="9" t="inlineStr"/>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="9" t="inlineStr"/>
     </row>
@@ -22778,11 +22806,7 @@
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr"/>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT ) ( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr"/>
     </row>
@@ -23055,7 +23079,11 @@
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr"/>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="9" t="inlineStr"/>
     </row>
@@ -23181,11 +23209,7 @@
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr"/>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I35" s="9" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr"/>
       <c r="K35" s="9" t="inlineStr"/>
     </row>
@@ -23228,7 +23252,11 @@
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr"/>
-      <c r="I36" s="9" t="inlineStr"/>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J36" s="9" t="inlineStr"/>
       <c r="K36" s="9" t="inlineStr"/>
     </row>
@@ -23354,11 +23382,7 @@
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr"/>
-      <c r="I39" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I39" s="9" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr"/>
       <c r="K39" s="9" t="inlineStr"/>
     </row>
@@ -23401,7 +23425,11 @@
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr"/>
-      <c r="I40" s="9" t="inlineStr"/>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J40" s="9" t="inlineStr"/>
       <c r="K40" s="9" t="inlineStr"/>
     </row>
@@ -23527,11 +23555,7 @@
         </is>
       </c>
       <c r="H43" s="11" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I43" s="9" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="9" t="inlineStr"/>
     </row>
@@ -23749,7 +23773,11 @@
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr"/>
-      <c r="I48" s="9" t="inlineStr"/>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J48" s="9" t="inlineStr"/>
       <c r="K48" s="9" t="inlineStr"/>
     </row>
@@ -23791,11 +23819,7 @@
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr"/>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I49" s="9" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr"/>
       <c r="K49" s="9" t="inlineStr"/>
     </row>
@@ -23838,7 +23862,11 @@
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr"/>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J50" s="9" t="inlineStr"/>
       <c r="K50" s="9" t="inlineStr"/>
     </row>
@@ -23922,7 +23950,11 @@
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr"/>
-      <c r="I52" s="9" t="inlineStr"/>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J52" s="9" t="inlineStr"/>
       <c r="K52" s="9" t="inlineStr"/>
     </row>
@@ -23964,11 +23996,7 @@
         </is>
       </c>
       <c r="H53" s="11" t="inlineStr"/>
-      <c r="I53" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I53" s="9" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr"/>
       <c r="K53" s="9" t="inlineStr"/>
     </row>
@@ -24140,7 +24168,11 @@
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr"/>
-      <c r="I57" s="9" t="inlineStr"/>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J57" s="9" t="inlineStr"/>
       <c r="K57" s="9" t="inlineStr"/>
     </row>
@@ -24342,11 +24374,7 @@
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr"/>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I62" s="9" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr"/>
       <c r="K62" s="9" t="inlineStr"/>
     </row>
@@ -24390,7 +24418,11 @@
         </is>
       </c>
       <c r="H63" s="11" t="inlineStr"/>
-      <c r="I63" s="9" t="inlineStr"/>
+      <c r="I63" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J63" s="9" t="inlineStr"/>
       <c r="K63" s="9" t="inlineStr"/>
     </row>
@@ -24646,11 +24678,7 @@
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr"/>
-      <c r="I69" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I69" s="9" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
       <c r="K69" s="9" t="inlineStr"/>
     </row>
@@ -24692,7 +24720,11 @@
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
-      <c r="I70" s="9" t="inlineStr"/>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J70" s="9" t="inlineStr"/>
       <c r="K70" s="9" t="inlineStr"/>
     </row>
@@ -24909,11 +24941,7 @@
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr"/>
-      <c r="I75" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I75" s="9" t="inlineStr"/>
       <c r="J75" s="9" t="inlineStr"/>
       <c r="K75" s="9" t="inlineStr"/>
     </row>
@@ -24949,7 +24977,11 @@
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
-      <c r="I76" s="9" t="inlineStr"/>
+      <c r="I76" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J76" s="9" t="inlineStr"/>
       <c r="K76" s="9" t="inlineStr"/>
     </row>
@@ -24985,11 +25017,7 @@
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr"/>
-      <c r="I77" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I77" s="9" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="9" t="inlineStr"/>
     </row>
@@ -25081,7 +25109,11 @@
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr"/>
-      <c r="I79" s="9" t="inlineStr"/>
+      <c r="I79" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J79" s="9" t="inlineStr"/>
       <c r="K79" s="9" t="inlineStr"/>
     </row>
@@ -25125,11 +25157,7 @@
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr"/>
-      <c r="I80" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I80" s="9" t="inlineStr"/>
       <c r="J80" s="9" t="inlineStr"/>
       <c r="K80" s="9" t="inlineStr"/>
     </row>
@@ -25174,7 +25202,11 @@
         </is>
       </c>
       <c r="H81" s="11" t="inlineStr"/>
-      <c r="I81" s="9" t="inlineStr"/>
+      <c r="I81" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J81" s="9" t="inlineStr"/>
       <c r="K81" s="9" t="inlineStr"/>
     </row>
@@ -25390,11 +25422,7 @@
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr"/>
-      <c r="I86" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I86" s="9" t="inlineStr"/>
       <c r="J86" s="9" t="inlineStr"/>
       <c r="K86" s="9" t="inlineStr"/>
     </row>
@@ -25430,7 +25458,11 @@
         </is>
       </c>
       <c r="H87" s="11" t="inlineStr"/>
-      <c r="I87" s="9" t="inlineStr"/>
+      <c r="I87" s="9" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
       <c r="J87" s="9" t="inlineStr"/>
       <c r="K87" s="9" t="inlineStr"/>
     </row>
@@ -26402,11 +26434,7 @@
         </is>
       </c>
       <c r="H114" s="11" t="inlineStr"/>
-      <c r="I114" s="9" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
+      <c r="I114" s="9" t="inlineStr"/>
       <c r="J114" s="9" t="inlineStr"/>
       <c r="K114" s="9" t="inlineStr"/>
     </row>
@@ -26554,7 +26582,11 @@
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr"/>
-      <c r="J4" s="16" t="inlineStr"/>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS DETERMINE THE MODE OF THE KNIFE HORIZONTAL ) ( POSITIONERS. ) ( )</t>
+        </is>
+      </c>
       <c r="K4" s="16" t="inlineStr"/>
     </row>
     <row r="5" ht="30" customHeight="1">
@@ -26881,7 +26913,7 @@
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -26908,16 +26940,8 @@
 |                                +-----+                 +-----+</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE AUTO AND MANUAL BLOWER SPEED INPUTS ARE SCALED TO 0-4095 IN THE ) ( CONFIGUATION FOR THE ANALOG INPUT CARD. ) ( )</t>
-        </is>
-      </c>
+      <c r="I4" s="13" t="inlineStr"/>
+      <c r="J4" s="13" t="inlineStr"/>
       <c r="K4" s="13" t="n">
         <v>0.966</v>
       </c>
@@ -26946,7 +26970,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -26973,16 +26997,8 @@
 |                                +-----+                 +-----+</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE NEXT GROUP OF RUNGS CONTROL INDICATOR LIGHTS. ) ( )</t>
-        </is>
-      </c>
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="13" t="inlineStr"/>
       <c r="K5" s="13" t="n">
         <v>0.977</v>
       </c>
@@ -27155,7 +27171,7 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>( ) ( DOWN SLOW ROTATION IS ALLOWED FROM 0 THRU 25 DEGREES, 170 THRU ) ( 205 DEGREES, 350 THRU 360 DEGREES OR ANYWHERE ABOVE MID-POSITION. ) ( )</t>
+          <t>( ) ( UP FAST ROTATION IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
         </is>
       </c>
       <c r="K8" s="13" t="n">
@@ -27186,7 +27202,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -27203,8 +27219,16 @@
 *       +-----------------------+</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
-      <c r="J9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( DOWN FAST IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
+        </is>
+      </c>
       <c r="K9" s="13" t="n">
         <v>0.8149999999999999</v>
       </c>
@@ -27257,7 +27281,7 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>( ) ( DOWN SLOW ROTATION IS ALLOWED FROM 0 THRU 25 DEGREES, 170 THRU 205 ) ( DEGREES, 350 THRU 360 DEGREES OR ANYWHERE ABOVE THE ELEVATOR ) ( MID-POSITION. ) ( )</t>
+          <t>( ) ( UP FAST IS ONLY ALLOWED ABOVE MID-POSITION WITH THE BAFFLES DISENGAGED. ) ( )</t>
         </is>
       </c>
       <c r="K10" s="13" t="n">
@@ -27288,7 +27312,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+</t>
+          <t>Wiring / constants differ;   -+--] [-----] [-----] [-----] [-----]/[-------------------------------------( )-- | ++--] [--+--] [-----] [-----] [--+--]/[-------------------------------------( )-- | +|       |                       | | +|       +-----------------------+; Comment text differs</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -27305,8 +27329,16 @@
 *       +-----------------------+</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
-      <c r="J11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( DOWN FAST IS ONLY ALLOWED ABOVE THE MID-POSITION WITH THE BAFFLES ) ( DISENGAGED. ) ( )</t>
+        </is>
+      </c>
       <c r="K11" s="13" t="n">
         <v>0.8149999999999999</v>
       </c>
@@ -27335,7 +27367,7 @@
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Outputs: ANAUTO, R401_12 → ANAUTO; Removed: %M00541, ENA_GAL, R401_12, SIMPKNA; Added: %M00093, %M00094, %M00095; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
@@ -27359,16 +27391,8 @@
 *--] [--+</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( Use Gap Auto to only allow movement if the correct mode from ACT ) ( is on. ) ( ) ( Skew mode, Passline mode (temp. disabled 3/24/17, ATM mode, ) ( and Z-Assist mode. ) ( )</t>
-        </is>
-      </c>
+      <c r="I12" s="13" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr"/>
       <c r="K12" s="13" t="n">
         <v>0.5659999999999999</v>
       </c>
@@ -27434,7 +27458,7 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>( ) ( Use height movement in Auto when ACT is in Height or Z-assist mode ) ( ) ( ) ( Use this timer to keep the Manual Request high for a time delay after ) ( swithcing back to auto. ) ( ) ( ) ( )</t>
+          <t>( ) ( Use Gap Auto to only allow movement if the correct mode from ACT ) ( is on. ) ( ) ( Skew mode, Passline mode (temp. disabled 3/24/17, ATM mode, ) ( and Z-Assist mode. ) ( )</t>
         </is>
       </c>
       <c r="K13" s="13" t="n">
@@ -27505,7 +27529,7 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>( ) ( Use this timer to pulse the moves for the knives in and out. ) ( This is to prevent overshoot and emulate how the operator ) ( bumps the knives in and out. ) ( ) ( ) ( Setpoint in 1st Timer, PULSEKN, %M0906 is the off delay (200 = 2secs) ) ( Setpoint in 2nd Timer, PULSKNR, %M0907 is the on time (25 = 250ms) ) ( )</t>
+          <t>( ) ( Use height movement in Auto when ACT is in Height or Z-assist mode ) ( ) ( ) ( Use this timer to keep the Manual Request high for a time delay after ) ( swithcing back to auto. ) ( ) ( ) ( )</t>
         </is>
       </c>
       <c r="K14" s="13" t="n">
@@ -27567,7 +27591,7 @@
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE FRONT ) ( HORIZONTAL POSITIONERS. ) ( )</t>
+          <t>( ) ( AUTO MODE INDICATOR LIGHT CONTROL RELAYS. ) ( )</t>
         </is>
       </c>
       <c r="K15" s="13" t="n">
@@ -27598,7 +27622,7 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
@@ -27637,8 +27661,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr"/>
-      <c r="J16" s="13" t="inlineStr"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE FRONT ) ( HORIZONTAL POSITIONERS. ) ( )</t>
+        </is>
+      </c>
       <c r="K16" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -27736,7 +27768,7 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
@@ -27763,16 +27795,8 @@
 *--] [-----] [----------+</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 1DR (FRONT KNIFE ) ( DRIVESIDE). ) ( )</t>
-        </is>
-      </c>
+      <c r="I18" s="13" t="inlineStr"/>
+      <c r="J18" s="13" t="inlineStr"/>
       <c r="K18" s="13" t="n">
         <v>0.968</v>
       </c>
@@ -27801,7 +27825,7 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
@@ -27840,8 +27864,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I19" s="13" t="inlineStr"/>
-      <c r="J19" s="13" t="inlineStr"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE OPERATOR SIDE FRONT ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K19" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -27870,7 +27902,7 @@
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
@@ -27909,16 +27941,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED SELECT FOR 2MTR (OPERATOR SIDE FRONT HORIZONTAL). ) ( )</t>
-        </is>
-      </c>
+      <c r="I20" s="13" t="inlineStr"/>
+      <c r="J20" s="13" t="inlineStr"/>
       <c r="K20" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -27981,7 +28005,7 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 2DR (OPERATOR SIDE FRONT ) ( KNIFE HORIZONTAL). ) ( )</t>
+          <t>( ) ( FAST SPEED SELECT FOR 2MTR (OPERATOR SIDE FRONT HORIZONTAL). ) ( )</t>
         </is>
       </c>
       <c r="K21" s="13" t="n">
@@ -28012,7 +28036,7 @@
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
@@ -28051,8 +28075,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
-      <c r="J22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE DRIVE SIDE REAR KNIFE ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K22" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -28081,7 +28113,7 @@
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -28120,16 +28152,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED CONTROL FOR 3MTR. ) ( )</t>
-        </is>
-      </c>
+      <c r="I23" s="13" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr"/>
       <c r="K23" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -28192,7 +28216,7 @@
       </c>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE THR INTERFACE RELAYS FOR 3DR. ) ( )</t>
+          <t>( ) ( FAST SPEED CONTROL FOR 3MTR. ) ( )</t>
         </is>
       </c>
       <c r="K24" s="13" t="n">
@@ -28223,7 +28247,7 @@
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
@@ -28262,8 +28286,16 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I25" s="13" t="inlineStr"/>
-      <c r="J25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( THE NEXT 2 RUNGS GENERATE REQUESTS FOR THE OPERATOR SIDE REAR KNIFE ) ( HORIZONTAL POSITIONER. ) ( )</t>
+        </is>
+      </c>
       <c r="K25" s="13" t="n">
         <v>0.947</v>
       </c>
@@ -28292,7 +28324,7 @@
       </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>Removed: SIMULAT; Ladder wiring or constants also differ; Comment text differs</t>
+          <t>Removed: SIMULAT; Ladder wiring or constants also differ</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr">
@@ -28331,16 +28363,8 @@
 *--] [-----] [--+</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J26" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( FAST SPEED CONTROL OF 4MTR. ) ( )</t>
-        </is>
-      </c>
+      <c r="I26" s="13" t="inlineStr"/>
+      <c r="J26" s="13" t="inlineStr"/>
       <c r="K26" s="13" t="n">
         <v>0.959</v>
       </c>
@@ -28403,7 +28427,7 @@
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>( ) ( THE NEXT 6 RUNGS ARE INTERFACE RELAYS FOR 4DR (REAR KNIFE OPERATOR ) ( SIDE HORIZONTAL POSITIONER). ) ( )</t>
+          <t>( ) ( FAST SPEED CONTROL OF 4MTR. ) ( )</t>
         </is>
       </c>
       <c r="K27" s="13" t="n">
@@ -28434,7 +28458,7 @@
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>Added: %M00541; Ladder wiring or constants also differ</t>
+          <t>Added: %M00541; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
@@ -28470,8 +28494,16 @@
 *--] [--+</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr"/>
-      <c r="J28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( STARTER FAULT INDICATOR LIGHT ON THE PUSHBUTTON PANEL. ) ( )</t>
+        </is>
+      </c>
       <c r="K28" s="13" t="n">
         <v>0.944</v>
       </c>
@@ -28531,7 +28563,7 @@
       </c>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>( ) ( WHEN A DISENGAGE PUSHBUTTON REQUEST IS SEEN IN AUTO MODE, AUTO MODE ) ( IS DISABLED (LOCKED OUT) UNTIL THE AUTO/MAN SELECTOR SWITCH IS TOGGLED ) ( OR A BAFFLE ENGAGE PUSHBUTTON IS PRESSED. BAFFLE REQUESTS FROM THE WELD ) ( TRACKING ARE IGNORED WHILE THIS RUNG IS TRUE. ) ( )</t>
+          <t>( ) ( RESET STARTER FAULTS ) ( )</t>
         </is>
       </c>
       <c r="K29" s="13" t="n">
@@ -28562,7 +28594,7 @@
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+; Comment text differs</t>
+          <t>Wiring / constants differ;   -|      +9.055000 +-----+       -6.099500 +-----+ | +|      +9.055000 +-----+       -5.099500 +-----+</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
@@ -28589,16 +28621,8 @@
 |      +9.055000 +-----+       -5.099500 +-----+</t>
         </is>
       </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>( COMMENT )</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>( ) ( Determine Skew of Top Knives ) ( ) ( ) ( Determine Top Side knife to Knife distance ) ( )</t>
-        </is>
-      </c>
+      <c r="I30" s="13" t="inlineStr"/>
+      <c r="J30" s="13" t="inlineStr"/>
       <c r="K30" s="13" t="n">
         <v>0.998</v>
       </c>
@@ -28765,7 +28789,7 @@
       <c r="I33" s="13" t="inlineStr"/>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>( ) ( ACT Appendix B: Section 5.1.2 ) ( ) ( R00436-440 Next Coating Weight Designation ) ( mapped from Wonderware at R00586-590 ) ( ) ( ) ( 3/14/17 ) ( %R436-440 was being overwritten due to being defined twice in wonderware ) ( so ) ( ACT changed to %R496-500 ) ( )</t>
+          <t>( ) ( ACT Appendix 3.2.k.1.0.x ) ( Knife Positions from ACT ) ( ) ( Permissive to move Knives in Auto. When in CLC Operatiing Mode, ACT ) ( controls the Pressure. Then if the oter modes, Z-Assist, Passline, ) ( Skew and ATM mode are selected, then the Knives can be moved ) ( automatically. ) ( ) ( )</t>
         </is>
       </c>
       <c r="K33" s="13" t="n">
@@ -28796,7 +28820,7 @@
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ</t>
+          <t>Outputs: SPTOPOP, TKO_SPA → TKO_SPA; Removed: SIMPKNA, SPTOPOP; Ladder wiring or constants also differ; Comment text differs</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr">
@@ -28823,8 +28847,16 @@
 |                +-----+</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
-      <c r="J34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( ACT Appendix B: Section 5.1.2 ) ( ) ( R00436-440 Next Coating Weight Designation ) ( mapped from Wonderware at R00586-590 ) ( ) ( ) ( 3/14/17 ) ( %R436-440 was being overwritten due to being defined twice in wonderware ) ( so ) ( ACT changed to %R496-500 ) ( )</t>
+        </is>
+      </c>
       <c r="K34" s="13" t="n">
         <v>0.5649999999999999</v>
       </c>
@@ -29024,7 +29056,7 @@
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |</t>
+          <t>Wiring / constants differ;   -|     +.02000000 | LEN |                      -.02000000 | LEN | | +|     +.01400000 | LEN |                      -.01400000 | LEN |; Comment text differs</t>
         </is>
       </c>
       <c r="G38" s="15" t="inlineStr">
@@ -29051,8 +29083,16 @@
 |                +-----+                                 +-----+</t>
         </is>
       </c>
-      <c r="I38" s="13" t="inlineStr"/>
-      <c r="J38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>( COMMENT )</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>( ) ( ) ( ) ( Auto Mode Parameters based on Setpoints from ACT ) ( ) ( ) ( )</t>
+        </is>
+      </c>
       <c r="K38" s="13" t="n">
         <v>0.992</v>
       </c>

</xml_diff>